<commit_message>
Frezyderm: refill supplemental descriptions/images
</commit_message>
<xml_diff>
--- a/frezyderm-catalog.xlsx
+++ b/frezyderm-catalog.xlsx
@@ -6278,7 +6278,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t xml:space="preserve">Frezyderm Holistic Calendula Cream 50ml</t>
+          <t xml:space="preserve">Frezyderm Holistic Calendula Cream, 50ml - Online Pharmacy Ofarmakopoiosmou.gr</t>
         </is>
       </c>
       <c r="B148">
@@ -6289,7 +6289,7 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t xml:space="preserve">Προϊόν Frezyderm — FREZYDERM Holistic Calendula Cream 50ml</t>
+          <t xml:space="preserve">Cream for face and body that relieves, moisturizes, soothes and helps balancing disorders of the skin flo</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
@@ -6304,7 +6304,12 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/calendula-cream-5202888261084.jpg</t>
+          <t xml:space="preserve">frezyderm/holistic-calendula-cream-50ml-online-pharmacy-ofarmakopoiosmou-gr-5202888261084.jpg</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ofarmakopoiosmou.gr/en/frezyderm-holistic-calendula-cream-50ml</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Frezyderm: sync official images
</commit_message>
<xml_diff>
--- a/frezyderm-catalog.xlsx
+++ b/frezyderm-catalog.xlsx
@@ -172,7 +172,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/aqua-care-gel-ph-7-50g-ofarmakopoiosmou-gr-5202888227554.jpg</t>
+          <t xml:space="preserve">frezyderm/aqua-care-gel-5202888227554.jpg</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -876,7 +876,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/acnorm-baby-40ml-pharm24-gr-5202888221224.jpg</t>
+          <t xml:space="preserve">frezyderm/ac-norm-baby-cream-5202888221224.jpg</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1882,7 +1882,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/active-sun-screen-tinted-face-cream-spf50-50ml-pharm24-gr-5202888400100.jpg</t>
+          <t xml:space="preserve">frezyderm/active-sun-screen-tinted-face-cream-spf-50-5202888400100.jpg</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/antidandruff-shampoo-for-oily-dandruff-200ml-online-pharmacy-ofarmakopoiosmou-gr-5202888105050.jpg</t>
+          <t xml:space="preserve">frezyderm/antidandruff-shampoo-5202888105050.jpg</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3719,7 +3719,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/baby-abcc-50ml-pharm24-gr-5202888101151.jpg</t>
+          <t xml:space="preserve">frezyderm/baby-a-b-c-c-5202888101151.jpg</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -3970,7 +3970,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/baby-cream-175ml-pharm24-gr-5202888221187.jpg</t>
+          <t xml:space="preserve">frezyderm/baby-cream-5202888221187.jpg</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -4024,7 +4024,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/baby-cream-50ml-pharm24-gr-5202888101076.jpg</t>
+          <t xml:space="preserve">frezyderm/baby-cream-5202888101076.jpg</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -4073,7 +4073,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/baby-foam-150ml-pharm24-gr-5202888101144.jpg</t>
+          <t xml:space="preserve">frezyderm/baby-foam-5202888101144.jpg</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -4433,7 +4433,7 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.frezyderm.gr/Images/f/ProductLarge//Content/Files/3D_PRODUCTS/Babyline/shampoo/BABY-SHAMPOO-300ml_700x963_01.jpg</t>
+          <t xml:space="preserve">frezyderm/baby-shampoo-5202888101069.jpg</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
@@ -4482,7 +4482,7 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/baby-shampoo-300ml-online-pharmacy-ofarmakopoiosmou-gr-5202888221248.png</t>
+          <t xml:space="preserve">frezyderm/baby-shampoo-5202888221248.jpg</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
@@ -4670,7 +4670,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/periodontitis-chlorhexene-0-2-gel-30ml-pharm24-gr-5202888281082.jpg</t>
+          <t xml:space="preserve">frezyderm/periodigum-chlorhexene-gel-5202888281082.jpg</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -5489,7 +5489,7 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/crilen-cream-50ml-pharm24-gr-5202888010989.jpg</t>
+          <t xml:space="preserve">frezyderm/crilen-5202888010989.jpg</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -6107,7 +6107,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/dmannosa-cranberry-extract-for-urinary-system-health-14x4gr-online-pharmacy-ofarmakopoiosm-5202888106200.jpg</t>
+          <t xml:space="preserve">frezyderm/dmannosa-5202888106200.jpg</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -6190,7 +6190,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/every-day-use-shampoo-200ml-online-pharmacy-ofarmakopoiosmou-gr-5202888105173.jpg</t>
+          <t xml:space="preserve">frezyderm/every-day-use-shampoo-5202888105173.jpg</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -6339,7 +6339,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/ferti-women-30-sachets-pharm24-gr-5202888331572.jpg</t>
+          <t xml:space="preserve">frezyderm/ferti-5202888331572.png</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -6748,7 +6748,7 @@
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/frezykeld-cream-40ml-pharm24-gr-5202888261008.jpg</t>
+          <t xml:space="preserve">frezyderm/frezykeld-cream-5202888261008.jpg</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
@@ -7613,7 +7613,7 @@
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/holistic-calendula-cream-50ml-online-pharmacy-ofarmakopoiosmou-gr-5202888261084.jpg</t>
+          <t xml:space="preserve">frezyderm/calendula-cream-5202888261084.jpg</t>
         </is>
       </c>
       <c r="K148" t="inlineStr">
@@ -8911,7 +8911,7 @@
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/intimeo-325mg-14caps-ofarmakopoiosmou-gr-5202888106194.jpg</t>
+          <t xml:space="preserve">frezyderm/intimeo-5202888106194.jpg</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -8962,7 +8962,7 @@
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/kids-sun-care-cream-spray-water-resistant-spf50-275ml-ofarmakopoiosmou-gr-5202888222450.jpg</t>
+          <t xml:space="preserve">frezyderm/kids-sun-care-cream-spray-spf-50-5202888222450.png</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -9236,7 +9236,7 @@
       </c>
       <c r="J179" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/for-kids-sun-nip-lotion-spf50-175ml-pharm24-gr-5202888222436.jpg</t>
+          <t xml:space="preserve">frezyderm/sun-screen-velvet-body-lotion-spf-50-5202888222436.jpg</t>
         </is>
       </c>
       <c r="K179" t="inlineStr">
@@ -9627,7 +9627,7 @@
       </c>
       <c r="J187" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.frezyderm.gr/Images/f/ProductLarge//Content/Files/3D_PRODUCTS/Hairline/mediated_shampoo/MEDIATED_SHAMPOO_200ml_700x963_01.jpg</t>
+          <t xml:space="preserve">frezyderm/mediated-shampoo-5202888105067.jpg</t>
         </is>
       </c>
       <c r="K187" t="inlineStr">
@@ -9729,7 +9729,7 @@
       </c>
       <c r="J189" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/mild-wash-foam-150ml-ofarmakopoiosmou-gr-5202888100123.png</t>
+          <t xml:space="preserve">frezyderm/mild-wash-foam-5202888100123.jpg</t>
         </is>
       </c>
       <c r="K189" t="inlineStr">
@@ -9835,7 +9835,7 @@
       </c>
       <c r="J191" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/moisturizing-24h-cream-20-50ml-pharm24-gr-5202888271007.jpg</t>
+          <t xml:space="preserve">frezyderm/moisturizing-24h-cream-5202888271007.jpg</t>
         </is>
       </c>
       <c r="K191" t="inlineStr">
@@ -9890,7 +9890,7 @@
       </c>
       <c r="J192" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/moisturizing-plus-cream-30-50ml-online-pharmacy-ofarmakopoiosmou-gr-5202888271014.png</t>
+          <t xml:space="preserve">frezyderm/moisturizing-plus-cream-5202888271014.jpg</t>
         </is>
       </c>
       <c r="K192" t="inlineStr">
@@ -9944,7 +9944,7 @@
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/moisturizing-rich-cream-45-dry-skin-50ml-online-pharmacy-ofarmakopoiosmou-gr-5202888271021.png</t>
+          <t xml:space="preserve">frezyderm/moisturizing-rich-cream-5202888271021.jpg</t>
         </is>
       </c>
       <c r="K193" t="inlineStr">
@@ -9997,7 +9997,7 @@
       </c>
       <c r="J194" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/gingivital-mouthwash-250ml-ofarmakopoiosmou-gr-5202888282027.jpg</t>
+          <t xml:space="preserve">frezyderm/gingivital-mouthwash-5202888282027.jpg</t>
         </is>
       </c>
       <c r="K194" t="inlineStr">
@@ -10151,7 +10151,7 @@
       </c>
       <c r="J197" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/periodigum-mouthwash-250ml-ofarmakopoiosmou-gr-5202888282010.jpg</t>
+          <t xml:space="preserve">frezyderm/periodigum-mouthwash-5202888282010.jpg</t>
         </is>
       </c>
       <c r="K197" t="inlineStr">
@@ -10659,7 +10659,7 @@
       </c>
       <c r="J207" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/night-force-a-e-cream-50ml-pharm24-gr-5202888271151.jpg</t>
+          <t xml:space="preserve">frezyderm/night-force-a-e-cream-5202888271151.jpg</t>
         </is>
       </c>
       <c r="K207" t="inlineStr">
@@ -11124,7 +11124,7 @@
       </c>
       <c r="J216" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/prelactic-gel-balancing-care-gel-50g-ofarmakopoiosmou-gr-5202888102899.jpg</t>
+          <t xml:space="preserve">frezyderm/prelactic-gel-5202888102899.jpg</t>
         </is>
       </c>
       <c r="K216" t="inlineStr">
@@ -11180,7 +11180,7 @@
       </c>
       <c r="J217" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.frezyderm.gr/Images/f/FacebookPresetSmall//Content/Files/3D_PRODUCTS/feminine/New_feminine_line_2024/Prevenstria/Prevenstria_frame1.jpg</t>
+          <t xml:space="preserve">frezyderm/prevenstria-protective-anti-stria-cream-5202888102110.jpg</t>
         </is>
       </c>
       <c r="K217" t="inlineStr">
@@ -11848,7 +11848,7 @@
       </c>
       <c r="J230" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/proflamine-40ml-pharm24-gr-5202888261015.jpg</t>
+          <t xml:space="preserve">frezyderm/proflamine-cream-5202888261015.jpg</t>
         </is>
       </c>
       <c r="K230" t="inlineStr">
@@ -11899,7 +11899,7 @@
       </c>
       <c r="J231" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/propolis-oral-spray-30ml-ofarmakopoiosmou-gr-5202888331022.jpg</t>
+          <t xml:space="preserve">frezyderm/propolis-oral-spray-5202888331022.jpg</t>
         </is>
       </c>
       <c r="K231" t="inlineStr">
@@ -12314,7 +12314,7 @@
       </c>
       <c r="J239" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/rectanal-aid-ointment-a-40ml-ofarmakopoiosmou-gr-5202888227592.png</t>
+          <t xml:space="preserve">frezyderm/rectanal-aid-ointment-5202888227592.jpg</t>
         </is>
       </c>
       <c r="K239" t="inlineStr">
@@ -12505,7 +12505,7 @@
       </c>
       <c r="J243" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/rinopure-sterile-isotonic-solution-of-sodium-chloride-0-9-30amps-x-5ml-online-pharmacy-ofa-5202888106217.jpg</t>
+          <t xml:space="preserve">frezyderm/rinopure-5202888106217.jpg</t>
         </is>
       </c>
       <c r="K243" t="inlineStr">
@@ -13050,7 +13050,7 @@
       </c>
       <c r="J254" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/sensitive-kids-face-body-milk-200ml-pharm24-gr-5202888230042.jpg</t>
+          <t xml:space="preserve">frezyderm/sensitive-kids-body-milk-5202888230042.jpg</t>
         </is>
       </c>
       <c r="K254" t="inlineStr">
@@ -13098,7 +13098,7 @@
       </c>
       <c r="J255" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/sensitive-kids-styling-gel-100ml-ofarmakopoiosmou-gr-5202888230073.jpg</t>
+          <t xml:space="preserve">frezyderm/sensitive-kids-styling-gel-5202888230073.jpg</t>
         </is>
       </c>
       <c r="K255" t="inlineStr">
@@ -15173,7 +15173,7 @@
       </c>
       <c r="J295" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/gingivital-toothpaste-1-000ppm-75ml-pharm24-gr-5202888281068.jpg</t>
+          <t xml:space="preserve">frezyderm/gingivital-toothpaste-5202888281068.jpg</t>
         </is>
       </c>
       <c r="K295" t="inlineStr">
@@ -15331,7 +15331,7 @@
       </c>
       <c r="J298" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/periodigum-toothpaste-75ml-pharm24-gr-5202888281044.jpg</t>
+          <t xml:space="preserve">frezyderm/periodigum-toothpaste-5202888281044.jpg</t>
         </is>
       </c>
       <c r="K298" t="inlineStr">
@@ -15439,7 +15439,7 @@
       </c>
       <c r="J300" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/pregnancy-toothpaste-75ml-online-pharmacy-ofarmakopoiosmou-gr-5202888281051.jpg</t>
+          <t xml:space="preserve">frezyderm/pregnancy-toothpaste-5202888281051.jpg</t>
         </is>
       </c>
       <c r="K300" t="inlineStr">
@@ -15962,7 +15962,7 @@
       </c>
       <c r="J310" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/vomi-free-30-chew-tabs-pharm24-gr-5202888331589.jpg</t>
+          <t xml:space="preserve">frezyderm/vomi-free-5202888331589.png</t>
         </is>
       </c>
       <c r="K310" t="inlineStr">

</xml_diff>